<commit_message>
Auto-cria config.json a partir de config_example.json se nao existir
</commit_message>
<xml_diff>
--- a/Fechamento/Apresentacao/Lista_Unidades.xlsx
+++ b/Fechamento/Apresentacao/Lista_Unidades.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DaVita\Projetos\0001 Fechamento\Apresentacao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alexandre\Repositorios\DaVita\Fechamento\Apresentacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B462996-2C43-466B-8660-28E3FDE28B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033ED566-9D41-41C5-A0A0-FD2E593C9E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79072CD0-1706-42D9-BB22-6128C78A0A93}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>unidade</t>
   </si>
@@ -184,6 +184,15 @@
   </si>
   <si>
     <t>DaVita Campo Grande</t>
+  </si>
+  <si>
+    <t>DaVita Campos</t>
+  </si>
+  <si>
+    <t>DaVita Contagem</t>
+  </si>
+  <si>
+    <t>DaVita Savassi</t>
   </si>
 </sst>
 </file>
@@ -252,8 +261,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}" name="Lista" displayName="Lista" ref="A1:C45" totalsRowShown="0">
-  <autoFilter ref="A1:C45" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}" name="Lista" displayName="Lista" ref="A1:C48" totalsRowShown="0">
+  <autoFilter ref="A1:C48" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{A09A0006-5E66-4F04-9B1B-91CF89EABDBF}" name="unidade"/>
     <tableColumn id="2" xr3:uid="{3E18FF90-D74A-4CB7-B418-92711F0D7D18}" name="mes " dataDxfId="2">
@@ -596,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F39A6D3-4A32-4BE2-A4C9-D1F4A3A6E4F5}">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
@@ -621,7 +630,7 @@
       </c>
       <c r="B2" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C2" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -634,7 +643,7 @@
       </c>
       <c r="B3" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C3" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -647,7 +656,7 @@
       </c>
       <c r="B4" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C4" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -660,7 +669,7 @@
       </c>
       <c r="B5" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C5" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -673,7 +682,7 @@
       </c>
       <c r="B6" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C6" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -686,7 +695,7 @@
       </c>
       <c r="B7" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C7" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -699,7 +708,7 @@
       </c>
       <c r="B8" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C8" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -712,7 +721,7 @@
       </c>
       <c r="B9" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C9" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -725,7 +734,7 @@
       </c>
       <c r="B10" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C10" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -738,7 +747,7 @@
       </c>
       <c r="B11" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C11" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -751,7 +760,7 @@
       </c>
       <c r="B12" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C12" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -764,7 +773,7 @@
       </c>
       <c r="B13" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C13" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -777,7 +786,7 @@
       </c>
       <c r="B14" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C14" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -790,7 +799,7 @@
       </c>
       <c r="B15" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C15" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -803,7 +812,7 @@
       </c>
       <c r="B16" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C16" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -816,7 +825,7 @@
       </c>
       <c r="B17" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C17" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -829,7 +838,7 @@
       </c>
       <c r="B18" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C18" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -842,7 +851,7 @@
       </c>
       <c r="B19" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C19" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -855,7 +864,7 @@
       </c>
       <c r="B20" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C20" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -868,7 +877,7 @@
       </c>
       <c r="B21" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C21" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -881,7 +890,7 @@
       </c>
       <c r="B22" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C22" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -894,7 +903,7 @@
       </c>
       <c r="B23" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C23" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -907,7 +916,7 @@
       </c>
       <c r="B24" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C24" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -920,7 +929,7 @@
       </c>
       <c r="B25" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C25" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -933,7 +942,7 @@
       </c>
       <c r="B26" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C26" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -946,7 +955,7 @@
       </c>
       <c r="B27" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C27" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -959,7 +968,7 @@
       </c>
       <c r="B28" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C28" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -972,7 +981,7 @@
       </c>
       <c r="B29" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C29" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -985,7 +994,7 @@
       </c>
       <c r="B30" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C30" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -998,7 +1007,7 @@
       </c>
       <c r="B31" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C31" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1011,7 +1020,7 @@
       </c>
       <c r="B32" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C32" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1024,7 +1033,7 @@
       </c>
       <c r="B33" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C33" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1037,7 +1046,7 @@
       </c>
       <c r="B34" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C34" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1050,7 +1059,7 @@
       </c>
       <c r="B35" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C35" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1063,7 +1072,7 @@
       </c>
       <c r="B36" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C36" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1076,7 +1085,7 @@
       </c>
       <c r="B37" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C37" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1089,7 +1098,7 @@
       </c>
       <c r="B38" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C38" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1102,7 +1111,7 @@
       </c>
       <c r="B39" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C39" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1115,7 +1124,7 @@
       </c>
       <c r="B40" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C40" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1128,7 +1137,7 @@
       </c>
       <c r="B41" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C41" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1141,7 +1150,7 @@
       </c>
       <c r="B42" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C42" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1154,7 +1163,7 @@
       </c>
       <c r="B43" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C43" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1167,7 +1176,7 @@
       </c>
       <c r="B44" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C44" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1180,9 +1189,48 @@
       </c>
       <c r="B45" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>abr</v>
+        <v>mai</v>
       </c>
       <c r="C45" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"aaaa")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"MMM")</f>
+        <v>mai</v>
+      </c>
+      <c r="C46" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"aaaa")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"MMM")</f>
+        <v>mai</v>
+      </c>
+      <c r="C47" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"aaaa")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"MMM")</f>
+        <v>mai</v>
+      </c>
+      <c r="C48" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
         <v>2026</v>
       </c>
@@ -1210,7 +1258,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(fechamento): atualiza lista de unidades
</commit_message>
<xml_diff>
--- a/Fechamento/Apresentacao/Lista_Unidades.xlsx
+++ b/Fechamento/Apresentacao/Lista_Unidades.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alexandre\Repositorios\DaVita\Fechamento\Apresentacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033ED566-9D41-41C5-A0A0-FD2E593C9E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A32BB7-B88A-413F-ADFA-E0B23F15EFE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79072CD0-1706-42D9-BB22-6128C78A0A93}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>unidade</t>
   </si>
@@ -193,6 +193,15 @@
   </si>
   <si>
     <t>DaVita Savassi</t>
+  </si>
+  <si>
+    <t>DaVita Mooca SH</t>
+  </si>
+  <si>
+    <t>DaVita Petrolina</t>
+  </si>
+  <si>
+    <t>DaVita Brotas</t>
   </si>
 </sst>
 </file>
@@ -261,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}" name="Lista" displayName="Lista" ref="A1:C48" totalsRowShown="0">
-  <autoFilter ref="A1:C48" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}" name="Lista" displayName="Lista" ref="A1:C51" totalsRowShown="0">
+  <autoFilter ref="A1:C51" xr:uid="{23667326-FEBA-4DD6-B322-122563FF40A0}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{A09A0006-5E66-4F04-9B1B-91CF89EABDBF}" name="unidade"/>
     <tableColumn id="2" xr3:uid="{3E18FF90-D74A-4CB7-B418-92711F0D7D18}" name="mes " dataDxfId="2">
@@ -605,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F39A6D3-4A32-4BE2-A4C9-D1F4A3A6E4F5}">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.7109375" bestFit="1" customWidth="1"/>
@@ -630,7 +639,7 @@
       </c>
       <c r="B2" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C2" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -643,7 +652,7 @@
       </c>
       <c r="B3" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C3" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -656,7 +665,7 @@
       </c>
       <c r="B4" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C4" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -669,7 +678,7 @@
       </c>
       <c r="B5" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C5" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -682,7 +691,7 @@
       </c>
       <c r="B6" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C6" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -695,7 +704,7 @@
       </c>
       <c r="B7" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C7" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -708,7 +717,7 @@
       </c>
       <c r="B8" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C8" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -721,7 +730,7 @@
       </c>
       <c r="B9" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C9" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -734,7 +743,7 @@
       </c>
       <c r="B10" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C10" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -747,7 +756,7 @@
       </c>
       <c r="B11" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C11" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -760,7 +769,7 @@
       </c>
       <c r="B12" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C12" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -773,7 +782,7 @@
       </c>
       <c r="B13" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C13" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -786,7 +795,7 @@
       </c>
       <c r="B14" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C14" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -799,7 +808,7 @@
       </c>
       <c r="B15" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C15" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -812,7 +821,7 @@
       </c>
       <c r="B16" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C16" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -825,7 +834,7 @@
       </c>
       <c r="B17" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C17" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -838,7 +847,7 @@
       </c>
       <c r="B18" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C18" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -851,7 +860,7 @@
       </c>
       <c r="B19" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C19" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -864,7 +873,7 @@
       </c>
       <c r="B20" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C20" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -877,7 +886,7 @@
       </c>
       <c r="B21" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C21" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -890,7 +899,7 @@
       </c>
       <c r="B22" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C22" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -903,7 +912,7 @@
       </c>
       <c r="B23" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C23" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -916,7 +925,7 @@
       </c>
       <c r="B24" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C24" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -929,7 +938,7 @@
       </c>
       <c r="B25" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C25" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -942,7 +951,7 @@
       </c>
       <c r="B26" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C26" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -955,7 +964,7 @@
       </c>
       <c r="B27" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C27" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -968,7 +977,7 @@
       </c>
       <c r="B28" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C28" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -981,7 +990,7 @@
       </c>
       <c r="B29" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C29" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -994,7 +1003,7 @@
       </c>
       <c r="B30" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C30" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1007,7 +1016,7 @@
       </c>
       <c r="B31" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C31" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1020,7 +1029,7 @@
       </c>
       <c r="B32" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C32" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1033,7 +1042,7 @@
       </c>
       <c r="B33" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C33" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1046,7 +1055,7 @@
       </c>
       <c r="B34" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C34" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1059,7 +1068,7 @@
       </c>
       <c r="B35" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C35" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1072,7 +1081,7 @@
       </c>
       <c r="B36" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C36" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1085,7 +1094,7 @@
       </c>
       <c r="B37" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C37" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1098,7 +1107,7 @@
       </c>
       <c r="B38" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C38" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1111,7 +1120,7 @@
       </c>
       <c r="B39" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C39" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1124,7 +1133,7 @@
       </c>
       <c r="B40" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C40" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1137,7 +1146,7 @@
       </c>
       <c r="B41" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C41" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1150,7 +1159,7 @@
       </c>
       <c r="B42" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C42" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1163,7 +1172,7 @@
       </c>
       <c r="B43" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C43" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1176,7 +1185,7 @@
       </c>
       <c r="B44" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C44" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1189,7 +1198,7 @@
       </c>
       <c r="B45" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C45" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1202,7 +1211,7 @@
       </c>
       <c r="B46" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C46" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1215,7 +1224,7 @@
       </c>
       <c r="B47" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C47" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
@@ -1228,9 +1237,48 @@
       </c>
       <c r="B48" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"MMM")</f>
-        <v>mai</v>
+        <v>jul</v>
       </c>
       <c r="C48" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"aaaa")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"MMM")</f>
+        <v>jul</v>
+      </c>
+      <c r="C49" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"aaaa")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"MMM")</f>
+        <v>jul</v>
+      </c>
+      <c r="C50" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"aaaa")</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="1" t="str">
+        <f>TEXT('Referencia'!$A$2,"MMM")</f>
+        <v>jul</v>
+      </c>
+      <c r="C51" s="1" t="str">
         <f>TEXT('Referencia'!$A$2,"aaaa")</f>
         <v>2026</v>
       </c>
@@ -1258,7 +1306,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>46143</v>
+        <v>46204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>